<commit_message>
Fix campo 7 stato fase length
</commit_message>
<xml_diff>
--- a/tests/fixtures/codici-test.xlsx
+++ b/tests/fixtures/codici-test.xlsx
@@ -413,7 +413,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD00001</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD0001</v>
       </c>
       <c r="B2" t="str">
         <v>ELENCO ELABORATI</v>
@@ -424,7 +424,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>RMB1284-ADD-RELGENERA-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-RELGENERA-XX-RT-Z-PD0001</v>
       </c>
       <c r="B3" t="str">
         <v>RELAZIONE GENERALE</v>
@@ -435,7 +435,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>RMB1284-ADD-PLANLIVEL-GF-DR-A-PD00001</v>
+        <v>RMB1284-ADD-PLANLIVEL-GF-DR-A-PD0001</v>
       </c>
       <c r="B4" t="str">
         <v>Rilievo Piano terra</v>
@@ -446,7 +446,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>RMB1284-ADD-PLANLIVEL-G1-DR-D-PD00001</v>
+        <v>RMB1284-ADD-PLANLIVEL-G1-DR-D-PD0001</v>
       </c>
       <c r="B5" t="str">
         <v>Demolizione selettiva Piano G1</v>
@@ -457,7 +457,7 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>RMB1284-ADD-PIASICCOO-XX-HS-D-PD00001</v>
+        <v>RMB1284-ADD-PIASICCOO-XX-HS-D-PD0001</v>
       </c>
       <c r="B6" t="str">
         <v>PSC</v>
@@ -468,7 +468,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>RMB1284-ADD-RELTECNIC-XX-RT-M-PD00005</v>
+        <v>RMB1284-ADD-RELTECNIC-XX-RT-M-PD0005</v>
       </c>
       <c r="B7" t="str">
         <v>Report di coordinamento (R1 update)</v>
@@ -523,7 +523,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>RMB1284-ADD-RELTECNIC-XX-RT-A-AN00099</v>
+        <v>RMB1284-ADD-RELTECNIC-XX-RT-A-AN0099</v>
       </c>
       <c r="B12" t="str">
         <v>Relazione As Built + Nuove costruzioni (composito)</v>
@@ -556,7 +556,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>RMB1284-ADM-RM0411001-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADM-RM0411001-XX-RT-Z-PD0001</v>
       </c>
       <c r="B15" t="str">
         <v>Codice Agenzia legacy ADM (Vulnerabilità Sismica)</v>
@@ -567,7 +567,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>RMB1284-ADD-PIPPOXXXX-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-PIPPOXXXX-XX-RT-Z-PD0001</v>
       </c>
       <c r="B16" t="str">
         <v>Codice documento sconosciuto 9 char</v>
@@ -578,7 +578,7 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>RMB1284-ADD-PLANGENER-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-PLANGENER-XX-RT-Z-PD0001</v>
       </c>
       <c r="B17" t="str">
         <v>PLANGENER (DR atteso) con RT</v>
@@ -589,10 +589,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD10001</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-P90001</v>
       </c>
       <c r="B18" t="str">
-        <v>Fase 1 (di norma 0)</v>
+        <v>Stato/Fase 9 non riconosciuto</v>
       </c>
       <c r="C18" t="str">
         <v>warning</v>
@@ -611,7 +611,7 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>RMB-ADD-RELGENERA-XX-RT-Z-PD00001</v>
+        <v>RMB-ADD-RELGENERA-XX-RT-Z-PD0001</v>
       </c>
       <c r="B20" t="str">
         <v>Codice Bene troppo corto</v>
@@ -622,7 +622,7 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>RMB1284-ADD-ELEVAZIONI-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-ELEVAZIONI-XX-RT-Z-PD0001</v>
       </c>
       <c r="B21" t="str">
         <v>ELEVAZIONI (10 char) — bug della v0 ora corretto</v>
@@ -633,7 +633,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>RMB1284-ADD-RELGENERA-XX-RT-9-PD00001</v>
+        <v>RMB1284-ADD-RELGENERA-XX-RT-9-PD0001</v>
       </c>
       <c r="B22" t="str">
         <v>Disciplina cifra</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>RMB1284-ADD-RELGENERA-99-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-RELGENERA-99-RT-Z-PD0001</v>
       </c>
       <c r="B25" t="str">
         <v>Livello 99 non in tabella</v>
@@ -677,7 +677,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD00000</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD0000</v>
       </c>
       <c r="B26" t="str">
         <v>Progressivo 00</v>
@@ -688,7 +688,7 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>RMB1284 -ADD-ELENCELAB-XX-AM-Z-PD00001</v>
+        <v>RMB1284 -ADD-ELENCELAB-XX-AM-Z-PD0001</v>
       </c>
       <c r="B27" t="str">
         <v>Spazi embedded (dovrebbero essere normalizzati)</v>
@@ -699,7 +699,7 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve"> RMB1284-ADD-RELGENERA-XX-RT-Z-PD00001 </v>
+        <v xml:space="preserve"> RMB1284-ADD-RELGENERA-XX-RT-Z-PD0001 </v>
       </c>
       <c r="B28" t="str">
         <v>Spazi leading/trailing</v>
@@ -710,7 +710,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>rmb1284-add-relgenera-xx-rt-z-pd00001</v>
+        <v>rmb1284-add-relgenera-xx-rt-z-pd0001</v>
       </c>
       <c r="B29" t="str">
         <v>Lowercase (deve essere uppercased)</v>
@@ -721,7 +721,7 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD00001-EXTRA</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD0001-EXTRA</v>
       </c>
       <c r="B30" t="str">
         <v>8 parti invece di 7</v>
@@ -757,7 +757,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD00001</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD0001</v>
       </c>
       <c r="C2" t="str">
         <v>ELENCO ELABORATI</v>
@@ -768,7 +768,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>RMB1284-ADD-RELGENERA-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-RELGENERA-XX-RT-Z-PD0001</v>
       </c>
       <c r="C3" t="str">
         <v>RELAZIONE GENERALE</v>
@@ -779,7 +779,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>RMB1284-ADD-PLANLIVEL-GF-DR-A-PD00001</v>
+        <v>RMB1284-ADD-PLANLIVEL-GF-DR-A-PD0001</v>
       </c>
       <c r="C4" t="str">
         <v>Rilievo Piano terra</v>
@@ -790,7 +790,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>RMB1284-ADD-PLANLIVEL-G1-DR-D-PD00001</v>
+        <v>RMB1284-ADD-PLANLIVEL-G1-DR-D-PD0001</v>
       </c>
       <c r="C5" t="str">
         <v>Demolizione selettiva Piano G1</v>
@@ -801,7 +801,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>RMB1284-ADD-PIASICCOO-XX-HS-D-PD00001</v>
+        <v>RMB1284-ADD-PIASICCOO-XX-HS-D-PD0001</v>
       </c>
       <c r="C6" t="str">
         <v>PSC</v>
@@ -812,7 +812,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>RMB1284-ADD-RELTECNIC-XX-RT-M-PD00005</v>
+        <v>RMB1284-ADD-RELTECNIC-XX-RT-M-PD0005</v>
       </c>
       <c r="C7" t="str">
         <v>Report di coordinamento (R1 update)</v>
@@ -867,7 +867,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>RMB1284-ADD-RELTECNIC-XX-RT-A-AN00099</v>
+        <v>RMB1284-ADD-RELTECNIC-XX-RT-A-AN0099</v>
       </c>
       <c r="C12" t="str">
         <v>Relazione As Built + Nuove costruzioni (composito)</v>
@@ -900,7 +900,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>RMB1284-ADM-RM0411001-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADM-RM0411001-XX-RT-Z-PD0001</v>
       </c>
       <c r="C15" t="str">
         <v>Codice Agenzia legacy ADM (Vulnerabilità Sismica)</v>
@@ -911,7 +911,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>RMB1284-ADD-PIPPOXXXX-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-PIPPOXXXX-XX-RT-Z-PD0001</v>
       </c>
       <c r="C16" t="str">
         <v>Codice documento sconosciuto 9 char</v>
@@ -922,7 +922,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>RMB1284-ADD-PLANGENER-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-PLANGENER-XX-RT-Z-PD0001</v>
       </c>
       <c r="C17" t="str">
         <v>PLANGENER (DR atteso) con RT</v>
@@ -933,10 +933,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD10001</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-P90001</v>
       </c>
       <c r="C18" t="str">
-        <v>Fase 1 (di norma 0)</v>
+        <v>Stato/Fase 9 non riconosciuto</v>
       </c>
     </row>
     <row r="19">
@@ -955,7 +955,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="str">
-        <v>RMB-ADD-RELGENERA-XX-RT-Z-PD00001</v>
+        <v>RMB-ADD-RELGENERA-XX-RT-Z-PD0001</v>
       </c>
       <c r="C20" t="str">
         <v>Codice Bene troppo corto</v>
@@ -966,7 +966,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="str">
-        <v>RMB1284-ADD-ELEVAZIONI-XX-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-ELEVAZIONI-XX-RT-Z-PD0001</v>
       </c>
       <c r="C21" t="str">
         <v>ELEVAZIONI (10 char) — bug della v0 ora corretto</v>
@@ -977,7 +977,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="str">
-        <v>RMB1284-ADD-RELGENERA-XX-RT-9-PD00001</v>
+        <v>RMB1284-ADD-RELGENERA-XX-RT-9-PD0001</v>
       </c>
       <c r="C22" t="str">
         <v>Disciplina cifra</v>
@@ -1010,7 +1010,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="str">
-        <v>RMB1284-ADD-RELGENERA-99-RT-Z-PD00001</v>
+        <v>RMB1284-ADD-RELGENERA-99-RT-Z-PD0001</v>
       </c>
       <c r="C25" t="str">
         <v>Livello 99 non in tabella</v>
@@ -1021,7 +1021,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD00000</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD0000</v>
       </c>
       <c r="C26" t="str">
         <v>Progressivo 00</v>
@@ -1032,7 +1032,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="str">
-        <v>RMB1284 -ADD-ELENCELAB-XX-AM-Z-PD00001</v>
+        <v>RMB1284 -ADD-ELENCELAB-XX-AM-Z-PD0001</v>
       </c>
       <c r="C27" t="str">
         <v>Spazi embedded (dovrebbero essere normalizzati)</v>
@@ -1043,7 +1043,7 @@
         <v>27</v>
       </c>
       <c r="B28" t="str">
-        <v xml:space="preserve"> RMB1284-ADD-RELGENERA-XX-RT-Z-PD00001 </v>
+        <v xml:space="preserve"> RMB1284-ADD-RELGENERA-XX-RT-Z-PD0001 </v>
       </c>
       <c r="C28" t="str">
         <v>Spazi leading/trailing</v>
@@ -1054,7 +1054,7 @@
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <v>rmb1284-add-relgenera-xx-rt-z-pd00001</v>
+        <v>rmb1284-add-relgenera-xx-rt-z-pd0001</v>
       </c>
       <c r="C29" t="str">
         <v>Lowercase (deve essere uppercased)</v>
@@ -1065,7 +1065,7 @@
         <v>29</v>
       </c>
       <c r="B30" t="str">
-        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD00001-EXTRA</v>
+        <v>RMB1284-ADD-ELENCELAB-XX-AM-Z-PD0001-EXTRA</v>
       </c>
       <c r="C30" t="str">
         <v>8 parti invece di 7</v>

</xml_diff>